<commit_message>
Publish Copenhagen_2021_WCH, Moscow_2021_MAR, Pitesti_2021_MAR, Szeged_2021_WC
</commit_message>
<xml_diff>
--- a/events/Moscow_2021_MAR/Moscow_2021_MAR_Results.xlsx
+++ b/events/Moscow_2021_MAR/Moscow_2021_MAR_Results.xlsx
@@ -2535,6 +2535,11 @@
           <t>00:15:20.800</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6796,6 +6801,11 @@
       <c r="P95" t="inlineStr">
         <is>
           <t>02:08:45.140</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>47779</t>
         </is>
       </c>
     </row>
@@ -9459,7 +9469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11662,6 +11672,28 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Kristina</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Bedec</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>